<commit_message>
Use generated sample files in the python-net docs
In the context of the GroupDocs.Watermark for Python via .NET 26.10
release. The sample files now come from GroupDocs.Watermark-SampleFiles,
which builds each one to contain what its examples look for and checks
it with the product.

- _sample_files: synced from the generator. 12 pages that linked
  flattened or parent-folder copies now link their own folder; the
  stale copies are removed.
- _output_files: regenerated, including the images-inside page;
  orphans under old paths removed.
- Snippets: the unprotect example opens protected-document.docx; the
  hyperlink-removal regex matches the sample's review link; the
  spreadsheet attachment examples skip linked attachments, which have
  no content.
- Prose: the PDF attachment listing and output sizes match the new
  files.
</commit_message>
<xml_diff>
--- a/python-net/_output_files/developer-guide/advanced-usage/adding-watermarks/add-watermarks-to-spreadsheet-documents/shapes-in-spreadsheet-document/remove_and_modify_shapes/output.xlsx
+++ b/python-net/_output_files/developer-guide/advanced-usage/adding-watermarks/add-watermarks-to-spreadsheet-documents/shapes-in-spreadsheet-document/remove_and_modify_shapes/output.xlsx
@@ -10,6 +10,9 @@
     <sheet name="Rate Card" sheetId="1" r:id="rId3"/>
     <sheet name="Project Budget" sheetId="2" r:id="rId4"/>
   </sheets>
+  <externalReferences>
+    <externalReference r:id="rId6"/>
+  </externalReferences>
   <definedNames/>
   <calcPr fullCalcOnLoad="1"/>
 </workbook>
@@ -329,6 +332,412 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr wrap="square"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr lang="en-US" u="none" baseline="0"/>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US"/>
+              <a:t>Budget by phase (USD)</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="6350">
+          <a:noFill/>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:v>Subtotal</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="3B7DD8"/>
+            </a:solidFill>
+            <a:effectLst/>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:cat>
+            <c:numRef>
+              <c:f>'Project Budget'!$A$5:$A$9</c:f>
+              <c:numCache>
+                <c:ptCount val="5"/>
+              </c:numCache>
+            </c:numRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Project Budget'!$D$5:$D$9</c:f>
+              <c:numCache>
+                <c:ptCount val="5"/>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:axId val="40197809"/>
+        <c:axId val="52809475"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="40197809"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6350" cap="flat" cmpd="sng"/>
+        </c:spPr>
+        <c:crossAx val="52809475"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="0"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="52809475"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350" cap="flat" cmpd="sng"/>
+            <a:effectLst/>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="out"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="6350" cap="flat" cmpd="sng"/>
+        </c:spPr>
+        <c:crossAx val="40197809"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:solidFill>
+          <a:srgbClr val="C0C0C0"/>
+        </a:solidFill>
+        <a:ln w="12700" cap="flat" cmpd="sng">
+          <a:solidFill>
+            <a:srgbClr val="808080"/>
+          </a:solidFill>
+        </a:ln>
+        <a:effectLst/>
+      </c:spPr>
+    </c:plotArea>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
+  </c:chart>
+</c:chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>12</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>666750</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>57150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp>
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="2" name="Validity note">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3dfad78f-9d8e-44b5-bd08-a82bfb782ce2}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="847725" y="2171700"/>
+          <a:ext cx="3429000" cy="381000"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:solidFill>
+          <a:srgbClr val="FFFFFF"/>
+        </a:solidFill>
+        <a:ln w="9525">
+          <a:solidFill>
+            <a:srgbClr val="000000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:style>
+        <a:lnRef idx="2">
+          <a:schemeClr val="accent1">
+            <a:shade val="50000"/>
+          </a:schemeClr>
+        </a:lnRef>
+        <a:fillRef idx="1">
+          <a:schemeClr val="accent1"/>
+        </a:fillRef>
+        <a:effectRef idx="0">
+          <a:schemeClr val="accent1"/>
+        </a:effectRef>
+        <a:fontRef idx="minor">
+          <a:schemeClr val="tx1"/>
+        </a:fontRef>
+      </xdr:style>
+      <xdr:txBody>
+        <a:bodyPr/>
+        <a:p>
+          <a:pPr/>
+          <a:r>
+            <a:rPr lang="en-US" u="none" baseline="0">
+              <a:solidFill>
+                <a:srgbClr val="5B6472"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>Rates valid until 31 December 2026. Prices exclude VAT.</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>371475</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>47625</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Aurora Visuals logo" descr="Aurora Visuals logo">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{2d54fb78-dca3-43f7-98c3-2031ed5d87e3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3609975" y="0"/>
+          <a:ext cx="1714500" cy="514350"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect"/>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="1" name="Budget by phase">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{3f797c09-03f1-4def-8cd1-7440ad6b6b02}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="2009775"/>
+        <a:ext cx="3733800" cy="2914650"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>6</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>7</xdr:col>
+          <xdr:colOff>533400</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>47625</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp>
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2050" name="Signed proposal" descr="northwind-proposal.docx" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2050"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{ef66ccde-d5ea-4b7c-9d52-f499f4399709}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr>
+              <a:spLocks noChangeAspect="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="4953000" y="628650"/>
+              <a:ext cx="1143000" cy="1428750"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect"/>
+            <a:noFill/>
+            <a:ln w="9525" cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+      <xdr:twoCellAnchor editAs="oneCell">
+        <xdr:from>
+          <xdr:col>9</xdr:col>
+          <xdr:colOff>0</xdr:colOff>
+          <xdr:row>3</xdr:row>
+          <xdr:rowOff>0</xdr:rowOff>
+        </xdr:from>
+        <xdr:to>
+          <xdr:col>10</xdr:col>
+          <xdr:colOff>533400</xdr:colOff>
+          <xdr:row>11</xdr:row>
+          <xdr:rowOff>47625</xdr:rowOff>
+        </xdr:to>
+        <xdr:sp>
+          <xdr:nvSpPr>
+            <xdr:cNvPr id="2051" name="Proposal PDF (linked)" descr="northwind-proposal.pdf" hidden="1">
+              <a:extLst>
+                <a:ext uri="{63B3BB69-23CF-44E3-9099-C40C66FF867C}">
+                  <a14:compatExt spid="_x0000_s2051"/>
+                </a:ext>
+                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{93d9c857-f085-42a4-a9bf-08b366f83b9f}"/>
+                </a:ext>
+              </a:extLst>
+            </xdr:cNvPr>
+            <xdr:cNvSpPr>
+              <a:spLocks noChangeAspect="1"/>
+            </xdr:cNvSpPr>
+          </xdr:nvSpPr>
+          <xdr:spPr>
+            <a:xfrm>
+              <a:off x="6781800" y="628650"/>
+              <a:ext cx="1143000" cy="1428750"/>
+            </a:xfrm>
+            <a:prstGeom prst="rect"/>
+            <a:noFill/>
+            <a:ln w="9525" cmpd="sng">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </xdr:spPr>
+        </xdr:sp>
+        <xdr:clientData/>
+      </xdr:twoCellAnchor>
+    </mc:Choice>
+    <mc:Fallback/>
+  </mc:AlternateContent>
+</xdr:wsDr>
+</file>
+
+<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <oleLink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1" progId="Acrobat Document">
+    <oleItems>
+      <oleItem name="'" advise="1" preferPic="1"/>
+    </oleItems>
+  </oleLink>
+</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -627,7 +1036,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{e9a1b0ce-ac0e-4995-a52f-3b1d278272ec}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A7F65045-2656-4CBA-9FAB-C83CE7CCBAA8}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -747,11 +1156,18 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter>
+    <oddHeader>&amp;L&amp;"Arial,Bold"Aurora Visuals — Rate Card&amp;C&amp;G&amp;RValid for 2026</oddHeader>
+    <oddFooter>&amp;Lauroravisuals.example&amp;RPage &amp;P of &amp;N</oddFooter>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+  <legacyDrawingHF r:id="rId2"/>
+  <picture r:id="rId3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{f6938347-c180-45ff-b775-f45fff9d0458}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42E6D097-40C4-4863-B42E-20875A1CBAA8}">
   <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="12.75"/>
   <cols>
@@ -872,5 +1288,59 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing r:id="rId1"/>
+  <legacyDrawing r:id="rId5"/>
+  <oleObjects>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Word.Document.12" dvAspect="DVASPECT_ICON" shapeId="2050" r:id="rId2">
+          <objectPr defaultSize="0" r:id="rId3">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>6</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>7</xdr:col>
+                <xdr:colOff>533400</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>47625</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Word.Document.12" dvAspect="DVASPECT_ICON" shapeId="2050" r:id="rId2"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+      <mc:Choice Requires="x14">
+        <oleObject progId="Acrobat Document" dvAspect="DVASPECT_ICON" link="[1]!''''" oleUpdate="OLEUPDATE_ALWAYS" shapeId="2051">
+          <objectPr defaultSize="0" r:id="rId4">
+            <anchor moveWithCells="1">
+              <from>
+                <xdr:col>9</xdr:col>
+                <xdr:colOff>0</xdr:colOff>
+                <xdr:row>3</xdr:row>
+                <xdr:rowOff>0</xdr:rowOff>
+              </from>
+              <to>
+                <xdr:col>10</xdr:col>
+                <xdr:colOff>533400</xdr:colOff>
+                <xdr:row>11</xdr:row>
+                <xdr:rowOff>47625</xdr:rowOff>
+              </to>
+            </anchor>
+          </objectPr>
+        </oleObject>
+      </mc:Choice>
+      <mc:Fallback>
+        <oleObject progId="Acrobat Document" dvAspect="DVASPECT_ICON" link="[1]!''''" oleUpdate="OLEUPDATE_ALWAYS" shapeId="2051"/>
+      </mc:Fallback>
+    </mc:AlternateContent>
+  </oleObjects>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update python-net docs for 26.10: outputs from the 26.10 wheel, installation and platform requirements, evaluation marks, preview callbacks and the AGENTS.md copy
</commit_message>
<xml_diff>
--- a/python-net/_output_files/developer-guide/advanced-usage/adding-watermarks/add-watermarks-to-spreadsheet-documents/shapes-in-spreadsheet-document/remove_and_modify_shapes/output.xlsx
+++ b/python-net/_output_files/developer-guide/advanced-usage/adding-watermarks/add-watermarks-to-spreadsheet-documents/shapes-in-spreadsheet-document/remove_and_modify_shapes/output.xlsx
@@ -401,11 +401,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="40197809"/>
-        <c:axId val="52809475"/>
+        <c:axId val="42966447"/>
+        <c:axId val="21692902"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="40197809"/>
+        <c:axId val="42966447"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -418,14 +418,14 @@
         <c:spPr>
           <a:ln w="6350" cap="flat" cmpd="sng"/>
         </c:spPr>
-        <c:crossAx val="52809475"/>
+        <c:crossAx val="21692902"/>
         <c:crosses val="autoZero"/>
         <c:auto val="0"/>
         <c:lblOffset val="100"/>
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="52809475"/>
+        <c:axId val="21692902"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -444,7 +444,7 @@
         <c:spPr>
           <a:ln w="6350" cap="flat" cmpd="sng"/>
         </c:spPr>
-        <c:crossAx val="40197809"/>
+        <c:crossAx val="42966447"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>